<commit_message>
Clear incorrect forProperty spreadsheet axiom
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1273,13 +1273,7 @@
           <t>If x is forProperty y, then x is defined or specified relative to the property y; informational descriptions of x may additionally be about y.</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>ssn:forProperty rdfs:range ssn:Property ;
-  rdfs:domain [ a owl:Class ; owl:unionOf ( bfo:SpecificallyDependentContinuant bfo:Function bfo:ProcessProfile cco:InformationContentEntity ) ] .
-[ a owl:ObjectProperty ; owl:propertyChainAxiom ( cco:described_by cco:is_about ) ] rdfs:subPropertyOf ssn:forProperty .</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>This allows real capabilities and qualities to be property-relative while reserving aboutness for information content entities.</t>

</xml_diff>

<commit_message>
Document sample representation property chains
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1504,7 +1504,8 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>sosa:hasSample rdfs:domain sosa:FeatureOfInterest ; rdfs:range sosa:Sample .</t>
+          <t>sosa:hasSample rdfs:domain sosa:FeatureOfInterest ; rdfs:range sosa:Sample .
+sosa:hasSample owl:propertyChainAxiom ( cco:ont00001873 bfo:BFO_0000084 ) .</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -1945,7 +1946,8 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>sosa:isSampleOf owl:inverseOf sosa:hasSample .</t>
+          <t>sosa:isSampleOf owl:inverseOf sosa:hasSample .
+sosa:isSampleOf owl:propertyChainAxiom ( bfo:BFO_0000101 cco:ont00001938 ) .</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Document inverse-side direct mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1304,7 +1304,8 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>ssn:hasDeployment owl:inverseOf ssn:deployedSystem .</t>
+          <t>ssn:hasDeployment owl:inverseOf ssn:deployedSystem .
+ssn:hasDeployment rdfs:subPropertyOf bfo:BFO_0000056 .</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1680,7 +1681,8 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>ssn:inDeployment owl:inverseOf ssn:deployedOnPlatform .</t>
+          <t>ssn:inDeployment owl:inverseOf ssn:deployedOnPlatform .
+ssn:inDeployment rdfs:subPropertyOf bfo:BFO_0000056 .</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1713,7 +1715,8 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>sosa:isActedOnBy owl:inverseOf sosa:actsOnProperty .</t>
+          <t>sosa:isActedOnBy owl:inverseOf sosa:actsOnProperty .
+sosa:isActedOnBy rdfs:subPropertyOf cco:ont00001886 .</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1913,7 +1916,8 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>sosa:isResultOf owl:inverseOf sosa:hasResult .</t>
+          <t>sosa:isResultOf owl:inverseOf sosa:hasResult .
+sosa:isResultOf rdfs:subPropertyOf cco:ont00001816 .</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -2013,7 +2017,8 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeByActuator owl:inverseOf sosa:madeActuation .</t>
+          <t>sosa:madeByActuator owl:inverseOf sosa:madeActuation .
+sosa:madeByActuator rdfs:subPropertyOf cco:ont00001833 .</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -2116,7 +2121,8 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeObservation owl:inverseOf sosa:madeBySensor .</t>
+          <t>sosa:madeObservation owl:inverseOf sosa:madeBySensor .
+sosa:madeObservation rdfs:subPropertyOf cco:ont00001787 .</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -2149,7 +2155,8 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeSampling owl:inverseOf sosa:madeBySampler .</t>
+          <t>sosa:madeSampling owl:inverseOf sosa:madeBySampler .
+sosa:madeSampling rdfs:subPropertyOf cco:ont00001787 .</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Align observes to forProperty
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -2226,12 +2226,12 @@
         <is>
           <t>sosa:observes rdfs:domain sosa:Sensor .
 sosa:observes rdfs:range ssn:Property .
-sosa:observes rdfs:subPropertyOf bfo:has_participant .</t>
+sosa:observes rdfs:subPropertyOf ssn:forProperty .</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>sosa:observes is a capability-level relation between a sensor and a property. It maps to bfo:has_participant as a conservative upper mapping, capturing that both entities participate in observation processes, without overcommitting to a more specific relation.</t>
+          <t>sosa:observes is a capability-level relation between a sensor and a property. It is retained as a subproperty of ssn:forProperty rather than mapped directly to bfo:has_participant, because the relation is property-directed rather than a direct process/participant relation.</t>
         </is>
       </c>
       <c r="G34" s="3" t="n"/>

</xml_diff>

<commit_message>
Correct hosts and implementedBy property chains
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1574,20 +1574,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>sosa:hosts owl:inverseOf sosa:isHostedBy .
-sosa:hosts rdfs:domain sosa:Platform .
-sosa:hosts rdfs:range [ a owl:Class ; owl:unionOf ( ssn:System sosa:Platform ) ] .
-sosa:hosts rdfs:subPropertyOf [ a owl:ObjectProperty ;
-  owl:propertyChainAxiom ( bfo:bearer_of bfo:has_realization bfo:has_participant )
-] .
-sosa:isHostedBy rdfs:subPropertyOf [ a owl:ObjectProperty ;
-  owl:propertyChainAxiom ( [ owl:inverseOf bfo:has_participant ] [ owl:inverseOf bfo:has_realization ] [ owl:inverseOf bfo:bearer_of ] )
-] .</t>
+          <t>sosa:hosts owl:propertyChainAxiom ( bfo:bearer_of bfo:has_realization bfo:has_participant ) .</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Hosting is best treated as role-mediated support that is realized in processes involving the hosted system, since physical attachment patterns vary and aren’t uniformly parthood.</t>
+          <t>Hosting is treated as role-mediated support realized in processes involving the hosted system. The mapping row states only the forward property-chain axiom relevant to sosa:hosts; domain and range assertions are intentionally excluded from the mapping.</t>
         </is>
       </c>
       <c r="G15" s="3" t="n"/>
@@ -1615,12 +1607,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>ssn:implementedBy rdfs:subPropertyOf [ owl:propertyChainAxiom ( [ owl:inverseOf cco:prescribed_by ] [ owl:inverseOf cco:agent_in ] ) ] .</t>
+          <t>ssn:implementedBy owl:propertyChainAxiom ( cco:ont00001942 cco:ont00001833 ) .</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>If an entity implements a procedure, then there exists a process prescribed by that procedure in which the entity participates as an agent.</t>
+          <t>If a procedure is implemented by an entity, then there exists a process prescribed by that procedure in which the entity participates as an agent. The chain uses the named inverse properties prescribes and has_agent rather than anonymous owl:inverseOf property expressions.</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
@@ -1782,12 +1774,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>sosa:isHostedBy owl:inverseOf sosa:hosts .</t>
+          <t>sosa:isHostedBy owl:propertyChainAxiom ( bfo:participates_in bfo:realizes bfo:inheres_in ) .</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:hosts; see sosa:hosts row.</t>
+          <t>isHostedBy is the inverse-side role-mediated hosting pattern. The property chain uses named inverse BFO relations directly rather than anonymous owl:inverseOf expressions.</t>
         </is>
       </c>
       <c r="G21" s="3" t="n"/>

</xml_diff>

<commit_message>
Clear terminal datatype placeholders
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -2409,14 +2409,10 @@
           <t>Associates a simple literal value with a result.</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>subPropertyOf owl:topDataProperty</t>
-        </is>
-      </c>
+      <c r="E2" s="4" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Simple results are represented as datatype values.</t>
+          <t>No more specific datatype-property mapping is asserted in this mapping. The prior owl:topDataProperty placeholder is intentionally not retained as an OWL axiom, because it is semantically redundant and may obscure later placement under a more specific datatype-property hierarchy.</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -2442,14 +2438,10 @@
           <t>The result time associates a temporal value with a result.</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>subPropertyOf owl:topDataProperty</t>
-        </is>
-      </c>
+      <c r="E3" s="4" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Result time is a datatype-valued temporal annotation.</t>
+          <t>No more specific datatype-property mapping is asserted in this mapping. The prior owl:topDataProperty placeholder is intentionally not retained as an OWL axiom, because it is semantically redundant and may obscure later placement under a more specific datatype-property hierarchy.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>

</xml_diff>

<commit_message>
Add provisional sample relationship mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -3724,7 +3724,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>sampling:RelationshipNature is a subclass of cco:InformationContentEntity because it is a generically dependent continuant that carries content about the type of relation between two sosa:Samples. It is not a specifically dependent continuant because SDCs inhere in independent continuants or processes, and a sampling:SampleRelationship is neither.</t>
+          <t>Provisional mapping for instance-data testing. RelationshipNature is treated as descriptive/information content identifying the nature of a reified sample relationship. This needs close review because the SOSA sample-relationship pattern models relation-like content through classes.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -3763,7 +3763,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>sampling:SampleRelationship is a subclass of cco:InformationContentEntity because it is a generically dependent continuant that encodes a relational fact between two sosa:Samples. It is not a specifically dependent continuant because SDCs inhere in independent continuants or processes, and a sampling:SampleRelationship is neither.</t>
+          <t>Provisional mapping for instance-data testing. SampleRelationship is treated as a reified descriptive/information-content structure about a relationship involving samples. The class restrictions are retained as SOSA structural constraints. This needs close review before release because the pattern may require a richer BFO/CCO treatment.</t>
         </is>
       </c>
       <c r="G6" s="3" t="n"/>

</xml_diff>

<commit_message>
Defer reasoner-unsafe system mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1436,15 +1436,10 @@
           <t>If an entity has_property a ssn:Property, then that ssn:Property either inheres in that entity (for bfo:SpecificallyDependentContinuant) or is an occurrent part of the relevant process (for bfo:ProcessProfile).</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>ssn:hasProperty rdfs:subPropertyOf bfo:bearer_of .
-ssn:hasProperty rdfs:subPropertyOf bfo:has_occurrent_part .</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>ssn:hasProperty must cover both bfo:SpecificallyDependentContinuant (which inhere in continuants via bfo:bearer_of) and bfo:ProcessProfile (which are occurrent parts of processes via bfo:has_occurrent_part), consistent with the Common Classes sheet treatment of ssn:Property as the union of these two BFO types.</t>
+          <t>Deferred after reasoner testing. The prior dual mapping to bfo:bearer_of and bfo:has_occurrent_part made ssn:hasProperty unsatisfiable under ELK, likely because one SOSA/SSN property was being placed under BFO relations with incompatible domain/range constraints. Do not implement this as a single dual subproperty mapping without a separate modeling review.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -2593,14 +2588,10 @@
           <t>Every ssn-system:BatteryLifetime is a BFO:Function that has a realization which is a StasisOfArtifactOperationality that has an occurrent part Power and is caused by a process realizing an Affordance prescribed by a CCO:ArtifactDesign.</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>subClassOf bfo:Function and bfo:has_realization some (cco:StasisOfArtifactOperationality and (bfo:has_occurrent_part some cco:Power) and (cco:caused_by some (bfo:Process and bfo:realizes some (cco:Affordance and cco:prescribed_by some cco:ArtifactDesign))))</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>BatteryLifetime is modeled as a function because it characterizes how long the battery can support system operation. The realization in operational stasis with power participation reflects that battery lifetime is manifested through continued energy provision.</t>
+          <t>Deferred after reasoner testing. The prior class mapping block made ssn-system:BatteryLifetime unsatisfiable under ELK when combined with SSN Systems, CCO, and SSN2BFO. This mapping needs a separate reasoner-safe modeling review before reintroduction.</t>
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
@@ -3056,14 +3047,10 @@
           <t>Every ssn-system:MeasurementRange is a BFO:Function that has a realization which is a sosa:Observation affected by a ssn:Stimulus prescribed by a CCO:ArtifactFunctionSpecification.</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>subClassOf bfo:Function and bfo:has_realization some (sosa:Observation and cco:is_affected_by some (ssn:Stimulus and cco:prescribed_by some cco:ArtifactFunctionSpecification))</t>
-        </is>
-      </c>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>MeasurementRange is modeled as a function because it describes what a system is able to do when operating correctly, and is realized in observation processes. The realization constraint ties the abstract range to concrete observations affected by stimuli and governed by functional specifications.</t>
+          <t>Deferred after reasoner testing. The prior class mapping block made ssn-system:MeasurementRange unsatisfiable under ELK when combined with SSN Systems, CCO, and SSN2BFO. This mapping needs a separate reasoner-safe modeling review before reintroduction.</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>

</xml_diff>

<commit_message>
Fix hasSystemProperty dependence direction
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -2917,12 +2917,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasSystemProperty rdfs:subPropertyOf bfo:specifically_depends_on .</t>
+          <t>ssn-system:hasSystemProperty rdfs:subPropertyOf bfo:specifically_depended_on_by .</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>SystemProperty instantiates a determinate–determinable pattern, where the property is a determinate refinement of a more general SystemCapability and specifically depends on it.</t>
+          <t>Directionality correction: the source relation runs from system capability x to system property y, while the intended dependence runs from y specifically depending on x. Therefore this object property maps to bfo:specifically_depended_on_by (BFO_0000194), the inverse of bfo:specifically_depends_on.</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>

</xml_diff>

<commit_message>
Fix operating and survival property dependence direction
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -2752,12 +2752,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasOperatingProperty rdfs:subPropertyOf bfo:specifically_depends_on .</t>
+          <t>ssn-system:hasOperatingProperty rdfs:subPropertyOf bfo:specifically_depended_on_by .</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>OperatingProperty is a determinate refinement of an OperatingRange and specifically depends on that range rather than directly on the system.</t>
+          <t>Directionality correction: the source relation runs from operating range x to operating property y, while the intended dependence runs from y specifically depending on x. Therefore this object property maps to bfo:specifically_depended_on_by (BFO_0000194), the inverse of bfo:specifically_depends_on.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -2818,12 +2818,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasSurvivalProperty rdfs:subPropertyOf bfo:specifically_depends_on .</t>
+          <t>ssn-system:hasSurvivalProperty rdfs:subPropertyOf bfo:specifically_depended_on_by .</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>If a survival range x hasSurvivalProperty y, then y is a property that refines or parameterizes that survival range.</t>
+          <t>Directionality correction: the source relation runs from survival range x to survival property y, while the intended dependence runs from y specifically depending on x. Therefore this object property maps to bfo:specifically_depended_on_by (BFO_0000194), the inverse of bfo:specifically_depends_on.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>

</xml_diff>

<commit_message>
Defer selected SSN Systems dependence mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -2750,14 +2750,10 @@
           <t>If an operating range x hasOperatingProperty y, then y is a property that refines or parameterizes that operating range.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>ssn-system:hasOperatingProperty rdfs:subPropertyOf bfo:specifically_depended_on_by .</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Directionality correction: the source relation runs from operating range x to operating property y, while the intended dependence runs from y specifically depending on x. Therefore this object property maps to bfo:specifically_depended_on_by (BFO_0000194), the inverse of bfo:specifically_depends_on.</t>
+          <t>Deferred active OWL mapping: intended semantics remain that if operating range x has operating property y, then y specifically depends on x. Direct OWL subproperty mapping to BFO_0000194 is deferred because HermiT diagnostics show selected direct BFO dependence mappings reduce satisfiability in the merged full-OWL profile. Intended finer-grained relation should be documented or implemented through rule/COMS architecture rather than active OWL rdfs:subPropertyOf for now.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -2816,14 +2812,10 @@
           <t>If a survival range hasSurvivalProperty y, then y is a property that refines or parameterizes that survival range and specifically depends on it.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>ssn-system:hasSurvivalProperty rdfs:subPropertyOf bfo:specifically_depended_on_by .</t>
-        </is>
-      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Directionality correction: the source relation runs from survival range x to survival property y, while the intended dependence runs from y specifically depending on x. Therefore this object property maps to bfo:specifically_depended_on_by (BFO_0000194), the inverse of bfo:specifically_depends_on.</t>
+          <t>Deferred active OWL mapping: intended semantics remain that if survival range x has survival property y, then y specifically depends on x. Direct OWL subproperty mapping to BFO_0000194 is deferred because HermiT diagnostics show selected direct BFO dependence mappings reduce satisfiability in the merged full-OWL profile. Intended finer-grained relation should be documented or implemented through rule/COMS architecture rather than active OWL rdfs:subPropertyOf for now.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -2915,14 +2907,10 @@
           <t>If a system capability x hasSystemProperty y, then y is a property that refines or parameterizes x and cannot exist independently of that capability.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>ssn-system:hasSystemProperty rdfs:subPropertyOf bfo:specifically_depended_on_by .</t>
-        </is>
-      </c>
+      <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Directionality correction: the source relation runs from system capability x to system property y, while the intended dependence runs from y specifically depending on x. Therefore this object property maps to bfo:specifically_depended_on_by (BFO_0000194), the inverse of bfo:specifically_depends_on.</t>
+          <t>Deferred active OWL mapping: intended semantics remain that if capability x has system property y, then y specifically depends on x. Direct OWL subproperty mapping to BFO_0000194 is deferred because HermiT diagnostics show selected direct BFO dependence mappings reduce satisfiability in the merged full-OWL profile. Intended finer-grained relation should be documented or implemented through rule/COMS architecture rather than active OWL rdfs:subPropertyOf for now.</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>

</xml_diff>

<commit_message>
Defer SurvivalRange class mapping
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -3403,14 +3403,10 @@
           <t>Every ssn-system:SurvivalRange is a BFO:Function that has a realization which is a BFO:Process caused by a process realizing an Affordance prescribed by a CCO:ArtifactDesign.</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>subClassOf bfo:Function and bfo:has_realization some (bfo:Process and cco:caused_by some (bfo:Process and bfo:realizes some (cco:Affordance and cco:prescribed_by some cco:ArtifactDesign)))</t>
-        </is>
-      </c>
+      <c r="E29" s="2" t="n"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>SurvivalRange is modeled as a function because it characterizes what conditions a system can endure without loss of operational integrity. Its realization through affordance-realizing processes reflects that survival is manifested through system–environment interaction.</t>
+          <t>Temporarily deferred active OWL class-expression mapping: intended semantics remain that SurvivalRange is a survival-oriented system range/capability profile. HermiT diagnostics identify SurvivalRange as a high-impact dependency in the mixed ssn:hasProperty / hasSurvivalProperty / non-sample sosa: context. This evaluation does not prove the mapping is semantically wrong; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
         </is>
       </c>
       <c r="G29" s="3" t="n"/>

</xml_diff>

<commit_message>
Defer input output property mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1370,14 +1370,10 @@
           <t>If a procedure has an input, then it has that input in the same sense as CCO hasInput.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>subPropertyOf cco:has_input</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="n"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Both relations connect a prescriptive item (procedure/algorithm) to the information it requires for execution.</t>
+          <t>Intended semantics remain that ssn:hasInput relates procedures to their inputs. Active OWL direct property mapping is temporarily deferred because HermiT diagnostics identify this mapping as a one-class reducer for ssn:Input in the mixed source-restriction / sosa:Procedure context. This evaluation does not prove the mapping is semantically wrong; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -1403,14 +1399,10 @@
           <t>If a procedure has an output, then it has that output in the same sense as CCO hasOutput.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>subPropertyOf cco:has_output</t>
-        </is>
-      </c>
+      <c r="E10" s="2" t="n"/>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Both relations connect a procedure to information produced by executing what it prescribes.</t>
+          <t>Intended semantics remain that ssn:hasOutput relates procedures to their outputs. Active OWL direct property mapping is temporarily deferred because HermiT diagnostics identify this mapping as a one-class reducer for ssn:Output in the mixed source-restriction / sosa:Procedure context. This evaluation does not prove the mapping is semantically wrong; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>

</xml_diff>

<commit_message>
Operationalize SSN Systems domain range mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -2736,10 +2736,15 @@
           <t>If an operating range x hasOperatingProperty y, then y is a property that refines or parameterizes that operating range.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>ssn-system:hasOperatingProperty rdfs:domain ssn-system:OperatingRange .
+ssn-system:hasOperatingProperty rdfs:range ssn-system:OperatingProperty .</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Deferred active OWL mapping: intended semantics remain that if operating range x has operating property y, then y specifically depends on x. Direct OWL subproperty mapping to BFO_0000194 is deferred because HermiT diagnostics show selected direct BFO dependence mappings reduce satisfiability in the merged full-OWL profile. Intended finer-grained relation should be documented or implemented through rule/COMS architecture rather than active OWL rdfs:subPropertyOf for now.</t>
+          <t>BFO dependence subproperty mapping remains deferred. OWL operationalization is provided by source-level domain/range typing: hasOperatingProperty has domain OperatingRange and range OperatingProperty. BFO dependence entailment is not active OWL in this branch; future rule/COMS treatment is paused/not implemented here.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -2798,10 +2803,15 @@
           <t>If a survival range hasSurvivalProperty y, then y is a property that refines or parameterizes that survival range and specifically depends on it.</t>
         </is>
       </c>
-      <c r="E11" s="2" t="n"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ssn-system:hasSurvivalProperty rdfs:domain ssn-system:SurvivalRange .
+ssn-system:hasSurvivalProperty rdfs:range ssn-system:SurvivalProperty .</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Deferred active OWL mapping: intended semantics remain that if survival range x has survival property y, then y specifically depends on x. Direct OWL subproperty mapping to BFO_0000194 is deferred because HermiT diagnostics show selected direct BFO dependence mappings reduce satisfiability in the merged full-OWL profile. Intended finer-grained relation should be documented or implemented through rule/COMS architecture rather than active OWL rdfs:subPropertyOf for now.</t>
+          <t>BFO dependence subproperty mapping remains deferred. OWL operationalization is provided by source-level domain/range typing: hasSurvivalProperty has domain SurvivalRange and range SurvivalProperty. BFO dependence entailment is not active OWL in this branch; future rule/COMS treatment is paused/not implemented here.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -2893,10 +2903,15 @@
           <t>If a system capability x hasSystemProperty y, then y is a property that refines or parameterizes x and cannot exist independently of that capability.</t>
         </is>
       </c>
-      <c r="E14" s="2" t="n"/>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>ssn-system:hasSystemProperty rdfs:domain ssn-system:SystemCapability .
+ssn-system:hasSystemProperty rdfs:range ssn-system:SystemProperty .</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Deferred active OWL mapping: intended semantics remain that if capability x has system property y, then y specifically depends on x. Direct OWL subproperty mapping to BFO_0000194 is deferred because HermiT diagnostics show selected direct BFO dependence mappings reduce satisfiability in the merged full-OWL profile. Intended finer-grained relation should be documented or implemented through rule/COMS architecture rather than active OWL rdfs:subPropertyOf for now.</t>
+          <t>BFO dependence subproperty mapping remains deferred. OWL operationalization is provided by source-level domain/range typing: hasSystemProperty has domain SystemCapability and range SystemProperty. BFO dependence entailment is not active OWL in this branch; future rule/COMS treatment is paused/not implemented here.</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>

</xml_diff>

<commit_message>
Reject Input Output CCO mapping rationale
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1367,13 +1367,13 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>If a procedure has an input, then it has that input in the same sense as CCO hasInput.</t>
+          <t>If a procedure hasInput y, then y is an input to that procedure.</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Intended semantics remain that ssn:hasInput relates procedures to their inputs. Active OWL direct property mapping is temporarily deferred because HermiT diagnostics identify this mapping as a one-class reducer for ssn:Input in the mixed source-restriction / sosa:Procedure context. This evaluation does not prove the mapping is semantically wrong; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
+          <t>Prior direct CCO mapping to cco:has_input is removed/rejected. The source relation is retained as an SSN relation between a Procedure and its Input; no active CCO property mapping is asserted.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -1396,13 +1396,13 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>If a procedure has an output, then it has that output in the same sense as CCO hasOutput.</t>
+          <t>If a procedure hasOutput y, then y is an output of that procedure.</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Intended semantics remain that ssn:hasOutput relates procedures to their outputs. Active OWL direct property mapping is temporarily deferred because HermiT diagnostics identify this mapping as a one-class reducer for ssn:Output in the mixed source-restriction / sosa:Procedure context. This evaluation does not prove the mapping is semantically wrong; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
+          <t>Prior direct CCO mapping to cco:has_output is removed/rejected. The source relation is retained as an SSN relation between a Procedure and its Output; no active CCO property mapping is asserted.</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>

</xml_diff>

<commit_message>
Add HermiT-clean source domain range axioms
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1137,12 +1137,14 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf cco:affects</t>
+          <t>sosa:actsOnProperty rdfs:domain sosa:Actuation .
+sosa:actsOnProperty rdfs:range sosa:ActuatableProperty .
+subPropertyOf cco:affects</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>sosa:actsOnProperty maps to cco:affects because an actuation acting on a property constitutes a causal influence on that property — the actuation makes a difference to the property's state, which is precisely what cco:affects captures.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Actuation and range sosa:ActuatableProperty. The existing CCO subproperty mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -1177,7 +1179,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>ssn:deployedOnPlatform maps to bfo:has_participant because the platform participates in the deployment process as the entity on which systems are installed or hosted.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:Deployment and range sosa:Platform. The existing BFO participant mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -1212,7 +1214,7 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>ssn:deployedSystem maps to bfo:has_participant because the deployed system participates in the deployment process as the primary entity being positioned or installed.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:Deployment and range ssn:System. The existing BFO participant mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
@@ -1247,7 +1249,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>ssn:detects maps to cco:is_affected_by because detection minimally requires that the stimulus makes a causal difference to the sensor. The stimulus affects the sensor's state, triggering a response, which is precisely what cco:is_affected_by captures.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sensor and range ssn:Stimulus. The existing CCO affected-by mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -1304,13 +1306,15 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>ssn:hasDeployment owl:inverseOf ssn:deployedSystem .
+          <t>ssn:hasDeployment rdfs:domain ssn:System .
+ssn:hasDeployment rdfs:range ssn:Deployment .
+ssn:hasDeployment owl:inverseOf ssn:deployedSystem .
 ssn:hasDeployment rdfs:subPropertyOf bfo:BFO_0000056 .</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Inverse of ssn:deployedSystem; see ssn:deployedSystem row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn:Deployment. Existing inverse and BFO continuant-part mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -1370,10 +1374,15 @@
           <t>If a procedure hasInput y, then y is an input to that procedure.</t>
         </is>
       </c>
-      <c r="E9" s="2" t="n"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>ssn:hasInput rdfs:domain sosa:Procedure .
+ssn:hasInput rdfs:range ssn:Input .</t>
+        </is>
+      </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Prior direct CCO mapping to cco:has_input is removed/rejected. The source relation is retained as an SSN relation between a Procedure and its Input; no active CCO property mapping is asserted.</t>
+          <t>Prior direct CCO mapping to cco:has_input remains removed/rejected. OWL operationalization is source-level domain/range typing: domain sosa:Procedure and range ssn:Input; no active CCO property mapping is asserted.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -1399,10 +1408,15 @@
           <t>If a procedure hasOutput y, then y is an output of that procedure.</t>
         </is>
       </c>
-      <c r="E10" s="2" t="n"/>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>ssn:hasOutput rdfs:domain sosa:Procedure .
+ssn:hasOutput rdfs:range ssn:Output .</t>
+        </is>
+      </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Prior direct CCO mapping to cco:has_output is removed/rejected. The source relation is retained as an SSN relation between a Procedure and its Output; no active CCO property mapping is asserted.</t>
+          <t>Prior direct CCO mapping to cco:has_output remains removed/rejected. OWL operationalization is source-level domain/range typing: domain sosa:Procedure and range ssn:Output; no active CCO property mapping is asserted.</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -1498,7 +1512,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>“Sample of” is fundamentally representational (intended to stand in for the feature of interest), and this is a conservative upper mapping to that representational pattern.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:FeatureOfInterest and range sosa:Sample. Existing property-chain mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -1533,7 +1547,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>ssn:hasSubSystem maps to bfo:has_continuant_part because subsystems are structural components of larger systems — they are material continuants that are parts of the larger material continuant that constitutes the system.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn:System. The existing BFO continuant-part mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>
@@ -1594,12 +1608,14 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>ssn:implementedBy owl:propertyChainAxiom ( cco:ont00001942 cco:ont00001833 ) .</t>
+          <t>ssn:implementedBy rdfs:domain sosa:Procedure .
+ssn:implementedBy rdfs:range ssn:System .
+ssn:implementedBy owl:propertyChainAxiom ( cco:ont00001942 cco:ont00001833 ) .</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>If a procedure is implemented by an entity, then there exists a process prescribed by that procedure in which the entity participates as an agent. The chain uses the named inverse properties prescribes and has_agent rather than anonymous owl:inverseOf property expressions.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Procedure and range ssn:System. Existing property-chain mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
@@ -1627,12 +1643,14 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>ssn:implements owl:inverseOf ssn:implementedBy .</t>
+          <t>ssn:implements rdfs:domain ssn:System .
+ssn:implements rdfs:range sosa:Procedure .
+ssn:implements owl:inverseOf ssn:implementedBy .</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Inverse of ssn:implementedBy; see ssn:implementedBy row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range sosa:Procedure. Existing inverse note remains unchanged.</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -1660,13 +1678,15 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>ssn:inDeployment owl:inverseOf ssn:deployedOnPlatform .
+          <t>ssn:inDeployment rdfs:domain sosa:Platform .
+ssn:inDeployment rdfs:range ssn:Deployment .
+ssn:inDeployment owl:inverseOf ssn:deployedOnPlatform .
 ssn:inDeployment rdfs:subPropertyOf bfo:BFO_0000056 .</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Inverse of ssn:deployedOnPlatform; see ssn:deployedOnPlatform row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Platform and range ssn:Deployment. Existing inverse and BFO continuant-part mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>
@@ -1694,13 +1714,15 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>sosa:isActedOnBy owl:inverseOf sosa:actsOnProperty .
+          <t>sosa:isActedOnBy rdfs:domain sosa:ActuatableProperty .
+sosa:isActedOnBy rdfs:range sosa:Actuation .
+sosa:isActedOnBy owl:inverseOf sosa:actsOnProperty .
 sosa:isActedOnBy rdfs:subPropertyOf cco:ont00001886 .</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:actsOnProperty; see sosa:actsOnProperty row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:ActuatableProperty and range sosa:Actuation. Existing inverse and CCO affected-by mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
@@ -1794,12 +1816,14 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>sosa:isObservedBy owl:inverseOf sosa:observes .</t>
+          <t>sosa:isObservedBy rdfs:domain sosa:ObservableProperty .
+sosa:isObservedBy rdfs:range sosa:Sensor .
+sosa:isObservedBy owl:inverseOf sosa:observes .</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:observes; see sosa:observes row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:ObservableProperty and range sosa:Sensor. Existing inverse note remains unchanged.</t>
         </is>
       </c>
       <c r="G22" s="3" t="n"/>
@@ -1862,12 +1886,12 @@
         <is>
           <t>ssn:isProxyFor rdf:type owl:ObjectProperty ;
   rdfs:domain ssn:Stimulus ;
-  rdfs:range ssn:Property .</t>
+  rdfs:range sosa:ObservableProperty .</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Because a stimulus does not itself carry or represent information, but instead gives rise to information that represents a property for sensing or inference.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:Stimulus and range sosa:ObservableProperty, following the imported source restriction on Stimulus.</t>
         </is>
       </c>
       <c r="G24" s="3" t="n"/>
@@ -1929,13 +1953,15 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>sosa:isSampleOf owl:inverseOf sosa:hasSample .
+          <t>sosa:isSampleOf rdfs:domain sosa:Sample .
+sosa:isSampleOf rdfs:range sosa:FeatureOfInterest .
+sosa:isSampleOf owl:inverseOf sosa:hasSample .
 sosa:isSampleOf owl:propertyChainAxiom ( bfo:BFO_0000101 cco:ont00001938 ) .</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:hasSample; see sosa:hasSample row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sample and range sosa:FeatureOfInterest. Existing inverse and property-chain mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G26" s="3" t="n"/>
@@ -1963,12 +1989,14 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf cco:agent_in</t>
+          <t>sosa:madeActuation rdfs:domain sosa:Actuator .
+sosa:madeActuation rdfs:range sosa:Actuation .
+subPropertyOf cco:agent_in</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Actuations are planned processes and actuators agents in those processes.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Actuator and range sosa:Actuation. The existing CCO agent-in mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G27" s="3" t="n"/>
@@ -1996,13 +2024,14 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeByActuator owl:inverseOf sosa:madeActuation .
+          <t>sosa:madeByActuator rdfs:domain sosa:Actuation .
+sosa:madeByActuator owl:inverseOf sosa:madeActuation .
 sosa:madeByActuator rdfs:subPropertyOf cco:ont00001833 .</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:madeActuation; see sosa:madeActuation row.</t>
+          <t>OWL operationalization adds only the HermiT-clean source-level domain typing: domain sosa:Actuation. The source-level range axiom sosa:madeByActuator rdfs:range sosa:Actuator is held back because HermiT testing identified it as the failing axiom; existing inverse and CCO has-agent mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G28" s="3" t="n"/>
@@ -2037,7 +2066,7 @@
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>sosa:madeBySampler maps to cco:has_agent because samplers are agents in sampling processes.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sampling and range sosa:Sampler. The existing CCO has-agent mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G29" s="3" t="n"/>
@@ -2072,7 +2101,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>sosa:madeBySensor maps to cco:has_agent because sensors function as agents in observation processes.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Observation and range sosa:Sensor. The existing CCO has-agent mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G30" s="3" t="n"/>
@@ -2100,13 +2129,15 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeObservation owl:inverseOf sosa:madeBySensor .
+          <t>sosa:madeObservation rdfs:domain sosa:Sensor .
+sosa:madeObservation rdfs:range sosa:Observation .
+sosa:madeObservation owl:inverseOf sosa:madeBySensor .
 sosa:madeObservation rdfs:subPropertyOf cco:ont00001787 .</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:madeBySensor; see sosa:madeBySensor row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sensor and range sosa:Observation. Existing inverse and CCO agent-in mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G31" s="3" t="n"/>
@@ -2134,13 +2165,15 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeSampling owl:inverseOf sosa:madeBySampler .
+          <t>sosa:madeSampling rdfs:domain sosa:Sampler .
+sosa:madeSampling rdfs:range sosa:Sampling .
+sosa:madeSampling owl:inverseOf sosa:madeBySampler .
 sosa:madeSampling rdfs:subPropertyOf cco:ont00001787 .</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Inverse of sosa:madeBySampler; see sosa:madeBySampler row.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sampler and range sosa:Sampling. Existing inverse and CCO agent-in mapping notes remain unchanged.</t>
         </is>
       </c>
       <c r="G32" s="3" t="n"/>
@@ -2166,10 +2199,15 @@
           <t>If a sosa:Observation observed_property a ssn:Property, then that ssn:Property is an input to that sosa:Observation.</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>sosa:observedProperty rdfs:domain sosa:Observation .
+sosa:observedProperty rdfs:range sosa:ObservableProperty .</t>
+        </is>
+      </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Intended semantics remain that observedProperty relates an observation to the observed property. Active OWL direct property mapping is temporarily deferred because HermiT diagnostics identify it as a narrow one-triple reducer for the remaining Observation / Sensor / Stimulus cluster. This evaluation does not prove the mapping is semantically wrong; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
+          <t>Prior direct CCO mapping to cco:has_input remains removed. OWL operationalization is source-level domain/range typing: domain sosa:Observation and range sosa:ObservableProperty; no active CCO property mapping is asserted.</t>
         </is>
       </c>
       <c r="G33" s="3" t="n"/>
@@ -2198,13 +2236,13 @@
       <c r="E34" s="2" t="inlineStr">
         <is>
           <t>sosa:observes rdfs:domain sosa:Sensor .
-sosa:observes rdfs:range ssn:Property .
+sosa:observes rdfs:range sosa:ObservableProperty .
 sosa:observes rdfs:subPropertyOf ssn:forProperty .</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>sosa:observes is a capability-level relation between a sensor and a property. It is retained as a subproperty of ssn:forProperty rather than mapped directly to bfo:has_participant, because the relation is property-directed rather than a direct process/participant relation.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sensor and range sosa:ObservableProperty. The existing ssn:forProperty mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G34" s="3" t="n"/>
@@ -2299,12 +2337,14 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf cco:process_started_by</t>
+          <t>ssn:wasOriginatedBy rdfs:domain sosa:Observation .
+ssn:wasOriginatedBy rdfs:range ssn:Stimulus .
+subPropertyOf cco:process_started_by</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Stimuli initiate observation processes.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Observation and range ssn:Stimulus. The existing CCO process-started-by mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G37" s="3" t="n"/>
@@ -2772,12 +2812,14 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasOperatingRange rdfs:subPropertyOf bfo:bearer_of .</t>
+          <t>ssn-system:hasOperatingRange rdfs:domain ssn:System .
+ssn-system:hasOperatingRange rdfs:range ssn-system:OperatingRange .
+ssn-system:hasOperatingRange rdfs:subPropertyOf bfo:bearer_of .</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>If a system x hasOperatingRange y, then y is an operating-range specification that inheres in x and characterizes the normal environmental conditions under which x is intended to operate.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn-system:OperatingRange. The existing BFO bearer relation mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -2839,12 +2881,14 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasSurvivalRange rdfs:subPropertyOf bfo:bearer_of .</t>
+          <t>ssn-system:hasSurvivalRange rdfs:domain ssn:System .
+ssn-system:hasSurvivalRange rdfs:range ssn-system:SurvivalRange .
+ssn-system:hasSurvivalRange rdfs:subPropertyOf bfo:bearer_of .</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>If a system x hasSurvivalRange y, then y is a survival-range specification that inheres in x and characterizes the conditions x can withstand without damage.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn-system:SurvivalRange. The existing BFO bearer relation mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
@@ -2872,12 +2916,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasSystemCapability rdfs:subPropertyOf bfo:bearer_of .</t>
+          <t>ssn-system:hasSystemCapability rdfs:domain ssn:System .
+ssn-system:hasSystemCapability rdfs:range ssn-system:SystemCapability .
+ssn-system:hasSystemCapability rdfs:subPropertyOf bfo:bearer_of .</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>SystemCapability is modeled as a specifically dependent continuant that inheres in the system as its bearer.</t>
+          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn-system:SystemCapability. The existing BFO bearer relation mapping remains unchanged.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>

</xml_diff>

<commit_message>
Defer SystemProperty direct class mapping
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -3543,17 +3543,13 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Every ssn-system:SystemProperty is either a BFO:SpecificallyDependentContinuant or a BFO:ProcessProfile that is prescribed by at least one CCO:ArtifactFunctionSpecification.</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>subClassOf (bfo:SpecificallyDependentContinuant or bfo:ProcessProfile) and cco:prescribed_by some cco:ArtifactFunctionSpecification</t>
-        </is>
-      </c>
+          <t>No direct active BFO/CCO class-expression mapping is asserted for ssn-system:SystemProperty; broader typing is inherited via ssn:Property.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>SystemProperty is treated as a specifically dependent continuant or process profile because it represents an intrinsic, dependent characteristic of a system’s functional behavior. The connection to ArtifactFunctionSpecification reflects that these properties are determined by functional design intent rather than empirical measurement alone.</t>
+          <t>Direct SystemProperty class-expression mapping deferred/removed. Broader target (specifically dependent continuant OR Process Profile) is inherited via ssn:Property. The prescribed_by some ArtifactFunctionSpecification branch is over-specific and not supported by imported ssn-systems.ttl source axioms. This change does not add sosa:madeByActuator rdfs:range sosa:Actuator and does not resolve the separate madeByActuator range redundancy discrepancy.</t>
         </is>
       </c>
       <c r="G32" s="3" t="n"/>

</xml_diff>

<commit_message>
Defer SOSA actuation agent property mappings
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1990,13 +1990,12 @@
       <c r="E27" s="2" t="inlineStr">
         <is>
           <t>sosa:madeActuation rdfs:domain sosa:Actuator .
-sosa:madeActuation rdfs:range sosa:Actuation .
-subPropertyOf cco:agent_in</t>
+sosa:madeActuation rdfs:range sosa:Actuation .</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Actuator and range sosa:Actuation. The existing CCO agent-in mapping remains unchanged.</t>
+          <t>OWL operationalization retains source-level domain/range typing: domain sosa:Actuator and range sosa:Actuation. Direct CCO agent-in mapping is deferred/removed as part of the paired actuation-agent deferral required for HermiT safety under the materialized SOSA import closure. This does not reject the intended agent semantics; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
         </is>
       </c>
       <c r="G27" s="3" t="n"/>
@@ -2025,13 +2024,12 @@
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>sosa:madeByActuator rdfs:domain sosa:Actuation .
-sosa:madeByActuator owl:inverseOf sosa:madeActuation .
-sosa:madeByActuator rdfs:subPropertyOf cco:ont00001833 .</t>
+sosa:madeByActuator owl:inverseOf sosa:madeActuation .</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization adds only the HermiT-clean source-level domain typing: domain sosa:Actuation. The source-level range axiom sosa:madeByActuator rdfs:range sosa:Actuator is held back because HermiT testing identified it as the failing axiom; existing inverse and CCO has-agent mapping notes remain unchanged.</t>
+          <t>OWL operationalization retains source-level domain typing: domain sosa:Actuation. Direct CCO has-agent mapping is deferred/removed as part of the paired actuation-agent deferral required for HermiT safety under the materialized SOSA import closure. This does not add sosa:madeByActuator rdfs:range sosa:Actuator and does not reject the intended agent semantics; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
         </is>
       </c>
       <c r="G28" s="3" t="n"/>

</xml_diff>

<commit_message>
Apply object property domain range minimal basis
</commit_message>
<xml_diff>
--- a/Current_SOSA-SSN to BFO-CCO.xlsx
+++ b/Current_SOSA-SSN to BFO-CCO.xlsx
@@ -1137,14 +1137,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>sosa:actsOnProperty rdfs:domain sosa:Actuation .
-sosa:actsOnProperty rdfs:range sosa:ActuatableProperty .
-subPropertyOf cco:affects</t>
+          <t>sosa:actsOnProperty rdfs:subPropertyOf cco:affects .</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Actuation and range sosa:ActuatableProperty. The existing CCO subproperty mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained sosa:isActedOnBy domain representative plus imported inverse/source axioms. Existing CCO subproperty mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G2" s="3" t="n"/>
@@ -1172,14 +1170,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>ssn:deployedOnPlatform rdfs:domain ssn:Deployment .
-ssn:deployedOnPlatform rdfs:range sosa:Platform .
-ssn:deployedOnPlatform rdfs:subPropertyOf bfo:has_participant .</t>
+          <t>ssn:deployedOnPlatform rdfs:subPropertyOf bfo:has_participant .</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:Deployment and range sosa:Platform. The existing BFO participant mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained ssn:inDeployment domain representative plus imported inverse/source axioms. Existing BFO participant mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G3" s="3" t="n"/>
@@ -1207,14 +1203,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>ssn:deployedSystem rdfs:domain ssn:Deployment .
-ssn:deployedSystem rdfs:range ssn:System .
-ssn:deployedSystem rdfs:subPropertyOf bfo:has_participant .</t>
+          <t>ssn:deployedSystem rdfs:subPropertyOf bfo:has_participant .</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:Deployment and range ssn:System. The existing BFO participant mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained ssn:hasDeployment domain representative plus imported inverse/source axioms. Existing BFO participant mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
@@ -1243,13 +1237,12 @@
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>ssn:detects rdfs:domain sosa:Sensor .
-ssn:detects rdfs:range ssn:Stimulus .
 ssn:detects rdfs:subPropertyOf cco:is_affected_by .</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sensor and range ssn:Stimulus. The existing CCO affected-by mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for ssn:detects and removes the local range assertion; the range typing remains entailed via the retained representative plus imported source restrictions. Existing CCO affected-by mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G5" s="3" t="n"/>
@@ -1307,14 +1300,13 @@
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>ssn:hasDeployment rdfs:domain ssn:System .
-ssn:hasDeployment rdfs:range ssn:Deployment .
 ssn:hasDeployment owl:inverseOf ssn:deployedSystem .
 ssn:hasDeployment rdfs:subPropertyOf bfo:BFO_0000056 .</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn:Deployment. Existing inverse and BFO continuant-part mapping notes remain unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for ssn:hasDeployment and removes the local range assertion; the inverse deployment typing remains entailed via retained representative plus imported/source inverse context. Existing inverse and BFO continuant-part mapping notes remain unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G7" s="3" t="n"/>
@@ -1376,13 +1368,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ssn:hasInput rdfs:domain sosa:Procedure .
-ssn:hasInput rdfs:range ssn:Input .</t>
+          <t>ssn:hasInput rdfs:domain sosa:Procedure .</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Prior direct CCO mapping to cco:has_input remains removed/rejected. OWL operationalization is source-level domain/range typing: domain sosa:Procedure and range ssn:Input; no active CCO property mapping is asserted.</t>
+          <t>Prior direct CCO mapping to cco:has_input remains removed/rejected. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; Input typing remains entailed via retained representative plus imported source restrictions. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -1410,13 +1401,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ssn:hasOutput rdfs:domain sosa:Procedure .
-ssn:hasOutput rdfs:range ssn:Output .</t>
+          <t>ssn:hasOutput rdfs:domain sosa:Procedure .</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Prior direct CCO mapping to cco:has_output remains removed/rejected. OWL operationalization is source-level domain/range typing: domain sosa:Procedure and range ssn:Output; no active CCO property mapping is asserted.</t>
+          <t>Prior direct CCO mapping to cco:has_output remains removed/rejected. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; Output typing remains entailed via retained representative plus imported source restrictions. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -1506,13 +1496,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>sosa:hasSample rdfs:domain sosa:FeatureOfInterest ; rdfs:range sosa:Sample .
-sosa:hasSample owl:propertyChainAxiom ( cco:ont00001873 bfo:BFO_0000084 ) .</t>
+          <t>sosa:hasSample owl:propertyChainAxiom ( cco:ont00001873 bfo:BFO_0000084 ) .</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:FeatureOfInterest and range sosa:Sample. Existing property-chain mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained sosa:isSampleOf domain representative plus imported inverse/source axioms. Existing property-chain mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -1541,13 +1530,12 @@
       <c r="E14" s="2" t="inlineStr">
         <is>
           <t>ssn:hasSubSystem rdfs:domain ssn:System .
-ssn:hasSubSystem rdfs:range ssn:System .
 ssn:hasSubSystem rdfs:subPropertyOf bfo:has_continuant_part .</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn:System. The existing BFO continuant-part mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; the range typing remains entailed via retained representative plus imported source restrictions. Existing BFO continuant-part mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>
@@ -1608,14 +1596,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>ssn:implementedBy rdfs:domain sosa:Procedure .
-ssn:implementedBy rdfs:range ssn:System .
-ssn:implementedBy owl:propertyChainAxiom ( cco:ont00001942 cco:ont00001833 ) .</t>
+          <t>ssn:implementedBy owl:propertyChainAxiom ( cco:ont00001942 cco:ont00001833 ) .</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Procedure and range ssn:System. Existing property-chain mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained ssn:implements domain representative plus imported inverse/source axioms. Existing property-chain mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G16" s="3" t="n"/>
@@ -1644,13 +1630,12 @@
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>ssn:implements rdfs:domain ssn:System .
-ssn:implements rdfs:range sosa:Procedure .
 ssn:implements owl:inverseOf ssn:implementedBy .</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range sosa:Procedure. Existing inverse note remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for ssn:implements and removes the local range assertion; the implementedBy/implements typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse note remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G17" s="3" t="n"/>
@@ -1679,14 +1664,13 @@
       <c r="E18" s="2" t="inlineStr">
         <is>
           <t>ssn:inDeployment rdfs:domain sosa:Platform .
-ssn:inDeployment rdfs:range ssn:Deployment .
 ssn:inDeployment owl:inverseOf ssn:deployedOnPlatform .
 ssn:inDeployment rdfs:subPropertyOf bfo:BFO_0000056 .</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Platform and range ssn:Deployment. Existing inverse and BFO continuant-part mapping notes remain unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for ssn:inDeployment and removes the local range assertion; deployedOnPlatform/inDeployment typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse and BFO continuant-part mapping notes remain unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>
@@ -1715,14 +1699,13 @@
       <c r="E19" s="2" t="inlineStr">
         <is>
           <t>sosa:isActedOnBy rdfs:domain sosa:ActuatableProperty .
-sosa:isActedOnBy rdfs:range sosa:Actuation .
 sosa:isActedOnBy owl:inverseOf sosa:actsOnProperty .
 sosa:isActedOnBy rdfs:subPropertyOf cco:ont00001886 .</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:ActuatableProperty and range sosa:Actuation. Existing inverse and CCO affected-by mapping notes remain unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for sosa:isActedOnBy and removes the local range assertion; actsOnProperty/isActedOnBy typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse and CCO affected-by mapping notes remain unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G19" s="3" t="n"/>
@@ -1817,13 +1800,12 @@
       <c r="E22" s="2" t="inlineStr">
         <is>
           <t>sosa:isObservedBy rdfs:domain sosa:ObservableProperty .
-sosa:isObservedBy rdfs:range sosa:Sensor .
 sosa:isObservedBy owl:inverseOf sosa:observes .</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:ObservableProperty and range sosa:Sensor. Existing inverse note remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for sosa:isObservedBy and removes the local range assertion; observes/isObservedBy typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse note remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G22" s="3" t="n"/>
@@ -1885,13 +1867,12 @@
       <c r="E24" s="2" t="inlineStr">
         <is>
           <t>ssn:isProxyFor rdf:type owl:ObjectProperty ;
-  rdfs:domain ssn:Stimulus ;
-  rdfs:range sosa:ObservableProperty .</t>
+  rdfs:domain ssn:Stimulus .</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:Stimulus and range sosa:ObservableProperty, following the imported source restriction on Stimulus.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; ObservableProperty typing remains entailed via retained representative plus imported source restrictions. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G24" s="3" t="n"/>
@@ -1954,14 +1935,13 @@
       <c r="E26" s="2" t="inlineStr">
         <is>
           <t>sosa:isSampleOf rdfs:domain sosa:Sample .
-sosa:isSampleOf rdfs:range sosa:FeatureOfInterest .
 sosa:isSampleOf owl:inverseOf sosa:hasSample .
 sosa:isSampleOf owl:propertyChainAxiom ( bfo:BFO_0000101 cco:ont00001938 ) .</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sample and range sosa:FeatureOfInterest. Existing inverse and property-chain mapping notes remain unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for sosa:isSampleOf and removes the local range assertion; hasSample/isSampleOf typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse and property-chain mapping notes remain unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G26" s="3" t="n"/>
@@ -1987,15 +1967,10 @@
           <t>If an actuation is made by an actuator, then the actuator is an agent participating in that actuation.</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>sosa:madeActuation rdfs:domain sosa:Actuator .
-sosa:madeActuation rdfs:range sosa:Actuation .</t>
-        </is>
-      </c>
+      <c r="E27" s="2" t="n"/>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization retains source-level domain/range typing: domain sosa:Actuator and range sosa:Actuation. Direct CCO agent-in mapping is deferred/removed as part of the paired actuation-agent deferral required for HermiT safety under the materialized SOSA import closure. This does not reject the intended agent semantics; future representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
+          <t>Direct CCO agent-in mapping remains deferred/removed as part of the paired actuation-agent deferral required for HermiT safety under the materialized SOSA import closure. Preferred cluster-minimal basis removes local domain/range assertions from this side; typing remains entailed via the retained sosa:madeByActuator domain representative plus imported inverse/source axioms. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G27" s="3" t="n"/>
@@ -2024,13 +1999,12 @@
       <c r="E28" s="2" t="inlineStr">
         <is>
           <t>sosa:madeByActuator rdfs:domain sosa:Actuation .
-sosa:madeByActuator rdfs:range sosa:Actuator .
 sosa:madeByActuator owl:inverseOf sosa:madeActuation .</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization now records source-level domain/range typing: domain sosa:Actuation and range sosa:Actuator. Direct CCO has-agent mapping remains deferred/removed as part of the paired actuation-agent deferral required for HermiT safety under the materialized SOSA import closure. This does not reject the intended agent semantics; future CCO/BFO agent representation should be reviewed for HermiT-safe OWL or rule/COMS treatment.</t>
+          <t>Direct CCO has-agent mapping remains deferred/removed as part of the paired actuation-agent deferral required for HermiT safety under the materialized SOSA import closure. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; Actuator typing remains entailed via retained representative plus imported inverse/source axioms. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G28" s="3" t="n"/>
@@ -2058,14 +2032,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeBySampler rdfs:domain sosa:Sampling .
-sosa:madeBySampler rdfs:range sosa:Sampler .
-sosa:madeBySampler rdfs:subPropertyOf cco:has_agent .</t>
+          <t>sosa:madeBySampler rdfs:subPropertyOf cco:has_agent .</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sampling and range sosa:Sampler. The existing CCO has-agent mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained sosa:madeSampling domain representative plus imported inverse/source axioms. Existing CCO has-agent mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G29" s="3" t="n"/>
@@ -2093,14 +2065,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>sosa:madeBySensor rdfs:domain sosa:Observation .
-sosa:madeBySensor rdfs:range sosa:Sensor .
-sosa:madeBySensor rdfs:subPropertyOf cco:has_agent .</t>
+          <t>sosa:madeBySensor rdfs:subPropertyOf cco:has_agent .</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Observation and range sosa:Sensor. The existing CCO has-agent mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained sosa:madeObservation domain representative plus imported inverse/source axioms. Existing CCO has-agent mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G30" s="3" t="n"/>
@@ -2129,14 +2099,13 @@
       <c r="E31" s="2" t="inlineStr">
         <is>
           <t>sosa:madeObservation rdfs:domain sosa:Sensor .
-sosa:madeObservation rdfs:range sosa:Observation .
 sosa:madeObservation owl:inverseOf sosa:madeBySensor .
 sosa:madeObservation rdfs:subPropertyOf cco:ont00001787 .</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sensor and range sosa:Observation. Existing inverse and CCO agent-in mapping notes remain unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for sosa:madeObservation and removes the local range assertion; madeObservation/madeBySensor typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse and CCO agent-in mapping notes remain unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G31" s="3" t="n"/>
@@ -2165,14 +2134,13 @@
       <c r="E32" s="2" t="inlineStr">
         <is>
           <t>sosa:madeSampling rdfs:domain sosa:Sampler .
-sosa:madeSampling rdfs:range sosa:Sampling .
 sosa:madeSampling owl:inverseOf sosa:madeBySampler .
 sosa:madeSampling rdfs:subPropertyOf cco:ont00001787 .</t>
         </is>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sampler and range sosa:Sampling. Existing inverse and CCO agent-in mapping notes remain unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative for sosa:madeSampling and removes the local range assertion; madeSampling/madeBySampler typing remains entailed via retained representative plus imported inverse/source axioms. Existing inverse and CCO agent-in mapping notes remain unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G32" s="3" t="n"/>
@@ -2200,13 +2168,12 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>sosa:observedProperty rdfs:domain sosa:Observation .
-sosa:observedProperty rdfs:range sosa:ObservableProperty .</t>
+          <t>sosa:observedProperty rdfs:domain sosa:Observation .</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Prior direct CCO mapping to cco:has_input remains removed. OWL operationalization is source-level domain/range typing: domain sosa:Observation and range sosa:ObservableProperty; no active CCO property mapping is asserted.</t>
+          <t>Prior direct CCO mapping to cco:has_input remains removed/rejected. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; ObservableProperty typing remains entailed via retained representative plus imported source restrictions. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G33" s="3" t="n"/>
@@ -2234,14 +2201,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>sosa:observes rdfs:domain sosa:Sensor .
-sosa:observes rdfs:range sosa:ObservableProperty .
-sosa:observes rdfs:subPropertyOf ssn:forProperty .</t>
+          <t>sosa:observes rdfs:subPropertyOf ssn:forProperty .</t>
         </is>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Sensor and range sosa:ObservableProperty. The existing ssn:forProperty mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis removes local domain/range assertions from this side of the inverse pair; the corresponding typing remains entailed via the retained sosa:isObservedBy domain representative plus imported inverse/source axioms. Existing ssn:forProperty mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G34" s="3" t="n"/>
@@ -2337,13 +2302,12 @@
       <c r="E37" s="2" t="inlineStr">
         <is>
           <t>ssn:wasOriginatedBy rdfs:domain sosa:Observation .
-ssn:wasOriginatedBy rdfs:range ssn:Stimulus .
-subPropertyOf cco:process_started_by</t>
+ssn:wasOriginatedBy rdfs:subPropertyOf cco:process_started_by .</t>
         </is>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain sosa:Observation and range ssn:Stimulus. The existing CCO process-started-by mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; Stimulus typing remains entailed via retained representative plus imported source restrictions. Existing CCO process-started-by mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G37" s="3" t="n"/>
@@ -2777,13 +2741,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasOperatingProperty rdfs:domain ssn-system:OperatingRange .
-ssn-system:hasOperatingProperty rdfs:range ssn-system:OperatingProperty .</t>
+          <t>ssn-system:hasOperatingProperty rdfs:domain ssn-system:OperatingRange .</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>BFO dependence subproperty mapping remains deferred. OWL operationalization is provided by source-level domain/range typing: hasOperatingProperty has domain OperatingRange and range OperatingProperty. BFO dependence entailment is not active OWL in this branch; future rule/COMS treatment is paused/not implemented here.</t>
+          <t>BFO dependence subproperty mapping remains deferred. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; OperatingProperty typing remains entailed via retained representative plus imported source restrictions. BFO dependence entailment is not active OWL in this branch. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G9" s="3" t="n"/>
@@ -2812,13 +2775,12 @@
       <c r="E10" s="2" t="inlineStr">
         <is>
           <t>ssn-system:hasOperatingRange rdfs:domain ssn:System .
-ssn-system:hasOperatingRange rdfs:range ssn-system:OperatingRange .
 ssn-system:hasOperatingRange rdfs:subPropertyOf bfo:bearer_of .</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn-system:OperatingRange. The existing BFO bearer relation mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; OperatingRange typing remains entailed via retained representative plus imported source restrictions. Existing BFO bearer relation mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -2846,13 +2808,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasSurvivalProperty rdfs:domain ssn-system:SurvivalRange .
-ssn-system:hasSurvivalProperty rdfs:range ssn-system:SurvivalProperty .</t>
+          <t>ssn-system:hasSurvivalProperty rdfs:domain ssn-system:SurvivalRange .</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>BFO dependence subproperty mapping remains deferred. OWL operationalization is provided by source-level domain/range typing: hasSurvivalProperty has domain SurvivalRange and range SurvivalProperty. BFO dependence entailment is not active OWL in this branch; future rule/COMS treatment is paused/not implemented here.</t>
+          <t>BFO dependence subproperty mapping remains deferred. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; SurvivalProperty typing remains entailed via retained representative plus imported source restrictions. BFO dependence entailment is not active OWL in this branch. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -2881,13 +2842,12 @@
       <c r="E12" s="2" t="inlineStr">
         <is>
           <t>ssn-system:hasSurvivalRange rdfs:domain ssn:System .
-ssn-system:hasSurvivalRange rdfs:range ssn-system:SurvivalRange .
 ssn-system:hasSurvivalRange rdfs:subPropertyOf bfo:bearer_of .</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn-system:SurvivalRange. The existing BFO bearer relation mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; SurvivalRange typing remains entailed via retained representative plus imported source restrictions. Existing BFO bearer relation mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
@@ -2916,13 +2876,12 @@
       <c r="E13" s="2" t="inlineStr">
         <is>
           <t>ssn-system:hasSystemCapability rdfs:domain ssn:System .
-ssn-system:hasSystemCapability rdfs:range ssn-system:SystemCapability .
 ssn-system:hasSystemCapability rdfs:subPropertyOf bfo:bearer_of .</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>OWL operationalization includes source-level domain/range typing: domain ssn:System and range ssn-system:SystemCapability. The existing BFO bearer relation mapping remains unchanged.</t>
+          <t>Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; SystemCapability typing remains entailed via retained representative plus imported source restrictions. Existing BFO bearer relation mapping remains unchanged. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G13" s="3" t="n"/>
@@ -2950,13 +2909,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>ssn-system:hasSystemProperty rdfs:domain ssn-system:SystemCapability .
-ssn-system:hasSystemProperty rdfs:range ssn-system:SystemProperty .</t>
+          <t>ssn-system:hasSystemProperty rdfs:domain ssn-system:SystemCapability .</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>BFO dependence subproperty mapping remains deferred. OWL operationalization is provided by source-level domain/range typing: hasSystemProperty has domain SystemCapability and range SystemProperty. BFO dependence entailment is not active OWL in this branch; future rule/COMS treatment is paused/not implemented here.</t>
+          <t>BFO dependence subproperty mapping remains deferred. Preferred cluster-minimal basis retains the explicit local domain representative and removes the local range assertion; SystemProperty typing remains entailed via retained representative plus imported source restrictions. BFO dependence entailment is not active OWL in this branch. Imported source axioms are untouched. This is not claimed as a globally exhaustive minimum.</t>
         </is>
       </c>
       <c r="G14" s="3" t="n"/>

</xml_diff>